<commit_message>
updated BOM with structural CF tubes
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\P01\P01_06_Procurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F4CC9F-9A32-417A-A458-F0BE5C60757F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7881D021-3687-4D17-80C4-788205B9752C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
+    <sheet name="Background_info" sheetId="2" r:id="rId1"/>
     <sheet name="Main_Table" sheetId="1" r:id="rId2"/>
     <sheet name="Totals" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="136">
   <si>
     <t>#</t>
   </si>
@@ -163,51 +163,12 @@
     <t>CF Tube 20x18mm</t>
   </si>
   <si>
-    <t>CF Tube 14x12mm</t>
-  </si>
-  <si>
-    <t>x600mm</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005010236031978.html?spm=a2g0o.productlist.main.6.b8402725vCj7PA&amp;algo_pvid=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a&amp;algo_exp_id=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a-5&amp;pdp_ext_f=%7B%22order%22%3A%22121%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2113.98%2113.80%21%21%21107.09%21105.71%21%40210156fc17817122154447423e1477%2112000051637131957%21sea%21BG%21892667464%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895%3BpisId%3A5000000205243253&amp;curPageLogUid=qunWAbdJt5rE&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010236031978%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
-    <t>10-22days</t>
-  </si>
-  <si>
-    <t>around 580mm needed per side</t>
-  </si>
-  <si>
-    <t>around 550mm needed per side</t>
-  </si>
-  <si>
-    <t>x250mm</t>
-  </si>
-  <si>
-    <t>9-17days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">around 180mm needed for the center </t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005010148436160.html?spm=a2g0o.productlist.main.39.b8402725vCj7PA&amp;algo_pvid=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a&amp;algo_exp_id=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a-36&amp;pdp_ext_f=%7B%22order%22%3A%22250%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%213.82%213.54%21%21%2129.28%2127.10%21%40210156fc17817122154447423e1477%2112000051321995472%21sea%21BG%21892667464%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=BGm65imvYIav&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010148436160%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
     <t>x1000mm</t>
   </si>
   <si>
-    <t>around 1000mm needed for the fuselage</t>
-  </si>
-  <si>
     <t>Delivery price (€)</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005010143347787.html?spm=a2g0o.productlist.main.55.b8402725vCj7PA&amp;algo_pvid=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a&amp;algo_exp_id=4d2bc5eb-91ce-454c-aea9-c9354bd4e78a-50&amp;pdp_ext_f=%7B%22order%22%3A%22410%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%219.24%219.06%21%21%2110.48%2110.28%21%40210156fc17817122154447423e1477%2112000051302007489%21sea%21BG%21892667464%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895%3BpisId%3A5000000205243253&amp;curPageLogUid=mLmDLRaNPLxT&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010143347787%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
-    <t>25days</t>
-  </si>
-  <si>
     <t>https://www.aliexpress.com/item/1005010143310151.html?spm=a2g0o.productlist.main.3.26867c47eNIIX8&amp;algo_pvid=a0a1c9bc-aaa9-43aa-905d-66f8a77d08a7&amp;algo_exp_id=a0a1c9bc-aaa9-43aa-905d-66f8a77d08a7-2&amp;pdp_ext_f=%7B%22order%22%3A%22230%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2138.62%2138.44%21%21%2143.80%2143.60%21%40212e508f17817230884093688e2c48%2112000051359404635%21sea%21BG%21892667464%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895%3BpisId%3A5000000204855994&amp;curPageLogUid=HADK0WdyQEtP&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010143310151%7C_p_origin_prod%3A</t>
   </si>
   <si>
@@ -226,13 +187,6 @@
     <t>6-10days</t>
   </si>
   <si>
-    <t>More than 1kg would be needed for the whole A/C.
-Order 1kg now and decide how to proceed after testing the material</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005002541518129.html?spm=a2g0o.productlist.main.5.78ffsq50sq503F&amp;algo_pvid=6faec72d-98e9-471e-b5a2-c2bb06b9fa94&amp;algo_exp_id=6faec72d-98e9-471e-b5a2-c2bb06b9fa94-4&amp;pdp_ext_f=%7B%22order%22%3A%221009%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2137.61%2130.33%21%21%2142.66%2134.40%21%40210319b017817235694855583e33c0%2112000033822258922%21sea%21BG%21892667464%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895%3BpisId%3A5000000209557399&amp;curPageLogUid=4m2AAUUDCr6v&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005002541518129%7C_p_origin_prod%3A</t>
-  </si>
-  <si>
     <t>1kg - White!</t>
   </si>
   <si>
@@ -440,10 +394,63 @@
     <t>Bearing come at 10 pcs</t>
   </si>
   <si>
-    <t>2x500mm needed for the outer wing senction</t>
-  </si>
-  <si>
     <t>https://3dprintx.bg/magazin/lw-pla-polylite-1-75-mm-0-8-kg-byal/?gad_source=1&amp;gad_campaignid=23369295043&amp;gbraid=0AAAABBeApTakpsbz_xdM7q_iQsCQTWH6b&amp;gclid=CjwKCAjw4dDTBhAqEiwAkHYmSltsrb_B0xt8ZKVKRAjDVP-SfQSydJNmmMURTd3Jy2valIBpp-DvshoC6SAQAvD_BwE</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005002433587874.html?spm=a2g0o.productlist.main.13.6b98nGcWnGcWLU&amp;algo_pvid=867aa278-ebeb-4d5e-84d7-d57d98923c8e&amp;algo_exp_id=867aa278-ebeb-4d5e-84d7-d57d98923c8e-12&amp;pdp_ext_f=%7B%22order%22%3A%22285%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2131.04%2131.05%21%21%2134.94%2134.94%21%400b0fe0e117862726418795124e0da9%2112000033609672339%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=4Gz3UoIpJ0b2&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005002433587874%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>Active foaming PLA-LW material.
+2 rolls of 1kg will be initially ordered.</t>
+  </si>
+  <si>
+    <t>around 820mm needed for each half-wing</t>
+  </si>
+  <si>
+    <t>CF Tube 18x16mm</t>
+  </si>
+  <si>
+    <t>around 550mm needed per side
+2 tubes per pack</t>
+  </si>
+  <si>
+    <t>x600mm (2 tubes per pack)</t>
+  </si>
+  <si>
+    <t>each</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005006436550237.html?spm=a2g0o.cart.0.0.730838dax88ROf&amp;mp=1&amp;pdp_npi=6%40dis%21EUR%21EUR+12.80%21EUR+12.80%21%21EUR+12.80%21%21%21%402103973d17862847051156158e10ad%2112000037159963415%21ct%21BG%21793291276%21%211%210%21</t>
+  </si>
+  <si>
+    <t>10-19days</t>
+  </si>
+  <si>
+    <t>full 1000mm length needed for each half-wing.
+2x944mm needed for structure inside fuselage.</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005006797742158.html?spm=a2g0o.cart.0.0.730838dax88ROf&amp;mp=1&amp;pdp_npi=6%40dis%21EUR%21EUR+26.70%21EUR+23.23%21%21EUR+23.23%21%21%21%402103973d17862847051156158e10ad%2112000038337169331%21ct%21BG%21793291276%21%211%210%21</t>
+  </si>
+  <si>
+    <t>10-20days</t>
+  </si>
+  <si>
+    <t>around 180mm needed for the center wing box
+around 550mm needed for each halfwing outbound
+4tubes per pack</t>
+  </si>
+  <si>
+    <t>x600mm (4 tubes per pack)</t>
+  </si>
+  <si>
+    <t>https://www.easycomposites.eu/6mm-woven-finish-carbon-fibre-tube</t>
+  </si>
+  <si>
+    <t>https://www.easycomposites.eu/22mm-woven-finish-carbon-fibre-tube</t>
+  </si>
+  <si>
+    <t>2-6 days</t>
   </si>
 </sst>
 </file>
@@ -513,7 +520,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,12 +536,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -593,7 +594,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -634,13 +635,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -656,28 +651,166 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="19">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC2EB15"/>
       <color rgb="FFFF8181"/>
     </mruColors>
   </colors>
@@ -1010,12 +1143,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1026,7 +1159,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -1037,7 +1170,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1048,7 +1181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1059,7 +1192,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1070,7 +1203,10 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>125</v>
+      </c>
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -1078,37 +1214,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1120,31 +1256,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:N33"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N38"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" style="7" customWidth="1"/>
-    <col min="3" max="3" width="57.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="8.85546875" style="1"/>
-    <col min="8" max="8" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" style="1"/>
+    <col min="2" max="2" width="37.6640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="57.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="5.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" style="1"/>
     <col min="13" max="13" width="48" style="17" customWidth="1"/>
-    <col min="14" max="16384" width="8.85546875" style="2"/>
+    <col min="14" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1161,7 +1297,7 @@
         <v>35</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>2</v>
@@ -1185,7 +1321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1217,12 +1353,12 @@
       <c r="K3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1231,7 +1367,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>29</v>
@@ -1249,249 +1385,254 @@
         <v>4</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="J4" s="15">
         <f>(G4*E4)+F4</f>
         <v>43.2</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="L4" s="18" t="s">
-        <v>10</v>
+        <v>44</v>
+      </c>
+      <c r="L4" s="28" t="s">
+        <v>36</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>41</v>
+        <v>122</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>42</v>
+        <v>124</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="15">
-        <v>8.65</v>
+        <v>12.8</v>
       </c>
       <c r="F5" s="15">
-        <v>0</v>
+        <v>5.16</v>
       </c>
       <c r="G5" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>43</v>
+        <v>125</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>126</v>
       </c>
       <c r="J5" s="15">
         <f>(G5*E5)+F5</f>
-        <v>17.3</v>
+        <v>17.96</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="L5" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M5" s="19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>42</v>
+        <v>132</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="15">
-        <v>10.199999999999999</v>
+        <v>23.23</v>
       </c>
       <c r="F6" s="15">
-        <v>0</v>
+        <v>10.09</v>
       </c>
       <c r="G6" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>43</v>
+        <v>125</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>129</v>
       </c>
       <c r="J6" s="15">
-        <f t="shared" ref="J6:J23" si="0">(G6*E6)+F6</f>
-        <v>20.399999999999999</v>
+        <f>(G6*E6)+F6</f>
+        <v>33.32</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="L6" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="L6" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M6" s="16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M6" s="19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="15">
-        <v>5.87</v>
-      </c>
-      <c r="F7" s="15">
-        <v>0</v>
+        <v>31.22</v>
+      </c>
+      <c r="F7" s="26">
+        <v>18.75</v>
       </c>
       <c r="G7" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="3" t="s">
-        <v>50</v>
+      <c r="I7" s="8" t="s">
+        <v>133</v>
       </c>
       <c r="J7" s="15">
-        <f t="shared" si="0"/>
-        <v>5.87</v>
-      </c>
-      <c r="K7" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" s="18" t="s">
+        <f t="shared" ref="J7:J21" si="0">(G7*E7)+F7</f>
+        <v>143.63</v>
+      </c>
+      <c r="K7" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="L7" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M7" s="19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="15">
-        <v>10.91</v>
-      </c>
-      <c r="F8" s="28">
-        <v>17.25</v>
-      </c>
+        <v>12.83</v>
+      </c>
+      <c r="F8" s="27"/>
       <c r="G8" s="15">
         <v>2</v>
       </c>
       <c r="H8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>54</v>
+      <c r="I8" s="8" t="s">
+        <v>134</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="0"/>
-        <v>39.07</v>
-      </c>
-      <c r="K8" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="L8" s="18" t="s">
+        <v>25.66</v>
+      </c>
+      <c r="K8" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="L8" s="28" t="s">
         <v>10</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E9" s="15">
-        <v>6</v>
-      </c>
-      <c r="F9" s="29"/>
+        <v>30.43</v>
+      </c>
+      <c r="F9" s="15">
+        <v>8.64</v>
+      </c>
       <c r="G9" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="15" t="s">
         <v>4</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>69.5</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="L9" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="L9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="M9" s="16"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M9" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="N9" s="25" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>40</v>
+      <c r="B10" s="20" t="s">
+        <v>50</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E10" s="15"/>
-      <c r="F10" s="26"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="15">
         <v>1</v>
       </c>
@@ -1499,298 +1640,302 @@
         <v>4</v>
       </c>
       <c r="I10" s="3"/>
-      <c r="J10" s="15"/>
+      <c r="J10" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="K10" s="15"/>
-      <c r="L10" s="18" t="s">
+      <c r="L10" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M10" s="16" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="M10" s="16"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>60</v>
+      <c r="B11" s="14" t="s">
+        <v>57</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E11" s="15">
-        <v>30.33</v>
+        <v>60.75</v>
       </c>
       <c r="F11" s="15">
-        <v>5.0599999999999996</v>
+        <v>0</v>
       </c>
       <c r="G11" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>4</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="0"/>
-        <v>35.39</v>
+        <v>243</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L11" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="L11" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M11" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="N11" s="30" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M11" s="16"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
         <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
         <v>10</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>65</v>
+      <c r="B12" s="14" t="s">
+        <v>105</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>65</v>
+        <v>103</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="E12" s="15">
+        <v>16.45</v>
+      </c>
+      <c r="F12" s="15">
+        <v>0</v>
+      </c>
       <c r="G12" s="15">
-        <v>1</v>
-      </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>104</v>
+      </c>
       <c r="J12" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K12" s="15"/>
-      <c r="L12" s="18" t="s">
+        <v>32.9</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L12" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M12" s="16"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M12" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="15">
         <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
         <v>11</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="15">
-        <v>60.75</v>
-      </c>
-      <c r="F13" s="15">
-        <v>0</v>
-      </c>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
       <c r="G13" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>88</v>
-      </c>
+      <c r="I13" s="3"/>
       <c r="J13" s="15">
         <f t="shared" si="0"/>
-        <v>243</v>
-      </c>
-      <c r="K13" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="L13" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="K13" s="15"/>
+      <c r="L13" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M13" s="16"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="15">
         <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
         <v>12</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>120</v>
+      <c r="B14" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="15">
-        <v>16.45</v>
-      </c>
-      <c r="F14" s="15">
-        <v>0</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I14" s="3" t="s">
-        <v>119</v>
-      </c>
+      <c r="I14" s="3"/>
       <c r="J14" s="15">
         <f t="shared" si="0"/>
-        <v>32.9</v>
-      </c>
-      <c r="K14" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L14" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="K14" s="15"/>
+      <c r="L14" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M14" s="16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M14" s="16"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="15">
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
         <v>13</v>
       </c>
       <c r="B15" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="13" t="s">
-        <v>67</v>
-      </c>
       <c r="D15" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="15">
+        <v>44.99</v>
+      </c>
+      <c r="F15" s="15">
         <v>19</v>
       </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
       <c r="G15" s="15">
-        <v>1</v>
-      </c>
-      <c r="H15" s="15"/>
-      <c r="I15" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="J15" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K15" s="15"/>
-      <c r="L15" s="18" t="s">
+        <v>198.96</v>
+      </c>
+      <c r="K15" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="L15" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M15" s="16"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="15">
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
         <v>14</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>73</v>
+      <c r="B16" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="E16" s="15">
+        <v>49.95</v>
+      </c>
+      <c r="F16" s="15">
+        <v>14.9</v>
+      </c>
       <c r="G16" s="15">
         <v>1</v>
       </c>
-      <c r="H16" s="15"/>
-      <c r="I16" s="3"/>
+      <c r="H16" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="J16" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K16" s="15"/>
-      <c r="L16" s="18" t="s">
+        <v>64.850000000000009</v>
+      </c>
+      <c r="K16" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="L16" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M16" s="16"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M16" s="16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="15">
         <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
         <v>15</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="13" t="s">
-        <v>86</v>
-      </c>
       <c r="D17" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="15">
-        <v>44.99</v>
-      </c>
-      <c r="F17" s="15">
-        <v>19</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
       <c r="G17" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I17" s="3" t="s">
-        <v>91</v>
-      </c>
+      <c r="I17" s="3"/>
       <c r="J17" s="15">
         <f t="shared" si="0"/>
-        <v>198.96</v>
-      </c>
-      <c r="K17" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="L17" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="K17" s="15"/>
+      <c r="L17" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M17" s="16"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
         <v>16</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E18" s="15">
-        <v>49.95</v>
+        <v>13.1</v>
       </c>
       <c r="F18" s="15">
-        <v>14.9</v>
+        <v>0</v>
       </c>
       <c r="G18" s="15">
         <v>1</v>
@@ -1799,69 +1944,81 @@
         <v>4</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="J18" s="15">
         <f t="shared" si="0"/>
-        <v>64.850000000000009</v>
+        <v>13.1</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="L18" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="L18" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="15">
         <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
         <v>17</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
+        <v>30</v>
+      </c>
+      <c r="E19" s="15">
+        <v>7.04</v>
+      </c>
+      <c r="F19" s="15">
+        <v>0</v>
+      </c>
       <c r="G19" s="15">
         <v>1</v>
       </c>
-      <c r="H19" s="15"/>
-      <c r="I19" s="3"/>
+      <c r="H19" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="J19" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K19" s="15"/>
-      <c r="L19" s="18" t="s">
+        <v>7.04</v>
+      </c>
+      <c r="K19" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L19" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M19" s="16"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M19" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="15">
         <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
         <v>18</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E20" s="15">
-        <v>13.1</v>
+        <v>14.81</v>
       </c>
       <c r="F20" s="15">
         <v>0</v>
@@ -1873,38 +2030,37 @@
         <v>4</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="0"/>
-        <v>13.1</v>
+        <v>14.81</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L20" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="15">
-        <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
         <v>19</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="15">
-        <v>7.04</v>
+        <v>6.61</v>
       </c>
       <c r="F21" s="15">
         <v>0</v>
@@ -1916,38 +2072,37 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="0"/>
-        <v>7.04</v>
+        <v>6.61</v>
       </c>
       <c r="K21" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L21" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="L21" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="15">
-        <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
-        <v>20</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>98</v>
+        <v>19</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>85</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="15">
-        <v>14.81</v>
+        <v>8.66</v>
       </c>
       <c r="F22" s="15">
         <v>0</v>
@@ -1958,78 +2113,70 @@
       <c r="H22" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I22" s="3" t="s">
-        <v>102</v>
+      <c r="I22" s="13" t="s">
+        <v>84</v>
       </c>
       <c r="J22" s="15">
-        <f t="shared" si="0"/>
-        <v>14.81</v>
+        <f t="shared" ref="J22:J27" si="1">(G22*E22)+F22</f>
+        <v>8.66</v>
       </c>
       <c r="K22" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L22" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="M22" s="16"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" s="15">
+        <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
+        <v>21</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="L22" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="M22" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
-        <v>19</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>106</v>
-      </c>
       <c r="C23" s="13" t="s">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="15">
-        <v>6.61</v>
-      </c>
-      <c r="F23" s="15">
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15">
+        <v>4</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I23" s="3"/>
+      <c r="J23" s="15">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G23" s="15">
-        <v>1</v>
-      </c>
-      <c r="H23" s="15"/>
-      <c r="I23" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J23" s="15">
-        <f t="shared" si="0"/>
-        <v>6.61</v>
-      </c>
-      <c r="K23" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L23" s="18" t="s">
+      <c r="K23" s="15"/>
+      <c r="L23" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M23" s="16" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M23" s="16"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="15">
-        <v>19</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>100</v>
+        <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
+        <v>22</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>93</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="E24" s="15">
-        <v>8.66</v>
+        <v>170.89</v>
       </c>
       <c r="F24" s="15">
         <v>0</v>
@@ -2040,68 +2187,80 @@
       <c r="H24" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="13" t="s">
-        <v>99</v>
+      <c r="I24" s="3" t="s">
+        <v>92</v>
       </c>
       <c r="J24" s="15">
-        <f t="shared" ref="J24:J29" si="1">(G24*E24)+F24</f>
-        <v>8.66</v>
+        <f t="shared" si="1"/>
+        <v>170.89</v>
       </c>
       <c r="K24" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="L24" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="L24" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M24" s="16"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M24" s="16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
       </c>
-      <c r="B25" s="23" t="s">
-        <v>76</v>
+      <c r="B25" s="13" t="s">
+        <v>66</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
+        <v>19</v>
+      </c>
+      <c r="E25" s="15">
+        <v>31.9</v>
+      </c>
+      <c r="F25" s="15">
+        <v>0</v>
+      </c>
       <c r="G25" s="15">
-        <v>4</v>
-      </c>
-      <c r="H25" s="15"/>
-      <c r="I25" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>31.9</v>
       </c>
       <c r="K25" s="15"/>
-      <c r="L25" s="18" t="s">
+      <c r="L25" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M25" s="16"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M25" s="16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>108</v>
+        <v>63</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E26" s="15">
-        <v>170.89</v>
+        <v>55.41</v>
       </c>
       <c r="F26" s="15">
         <v>0</v>
@@ -2113,306 +2272,290 @@
         <v>4</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v>170.89</v>
+        <v>55.41</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="L26" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="L26" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="15">
         <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
         <v>25</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E27" s="15">
-        <v>31.9</v>
-      </c>
-      <c r="F27" s="15">
-        <v>0</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
       <c r="G27" s="15">
         <v>1</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I27" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="I27" s="3"/>
       <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v>31.9</v>
+        <v>0</v>
       </c>
       <c r="K27" s="15"/>
-      <c r="L27" s="18" t="s">
+      <c r="L27" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M27" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M27" s="16"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="15">
         <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
         <v>26</v>
       </c>
-      <c r="B28" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>79</v>
+      <c r="B28" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>108</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="15">
-        <v>55.41</v>
-      </c>
-      <c r="F28" s="15">
-        <v>0</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E28" s="24">
+        <v>6.99</v>
+      </c>
+      <c r="F28" s="15"/>
       <c r="G28" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I28" s="3" t="s">
-        <v>113</v>
+      <c r="I28" s="23" t="s">
+        <v>111</v>
       </c>
       <c r="J28" s="15">
-        <f t="shared" si="1"/>
-        <v>55.41</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="L28" s="18" t="s">
+        <f t="shared" ref="J28" si="2">(G28*E28)+F28</f>
+        <v>27.96</v>
+      </c>
+      <c r="K28" s="15"/>
+      <c r="L28" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="M28" s="16" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M28" s="16"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="15">
         <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
         <v>27</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>87</v>
+      <c r="B29" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>109</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="15"/>
+      <c r="E29" s="15">
+        <v>7.19</v>
+      </c>
       <c r="F29" s="15"/>
       <c r="G29" s="15">
-        <v>1</v>
-      </c>
-      <c r="H29" s="15"/>
-      <c r="I29" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>110</v>
+      </c>
       <c r="J29" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" ref="J29" si="3">(G29*E29)+F29</f>
+        <v>14.38</v>
       </c>
       <c r="K29" s="15"/>
-      <c r="L29" s="18" t="s">
+      <c r="L29" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M29" s="16"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="15">
         <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
         <v>28</v>
       </c>
-      <c r="B30" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C30" s="24" t="s">
-        <v>123</v>
+      <c r="B30" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>109</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="27">
-        <v>6.99</v>
+      <c r="E30" s="15">
+        <v>7.19</v>
       </c>
       <c r="F30" s="15"/>
       <c r="G30" s="15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H30" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I30" s="25" t="s">
-        <v>126</v>
+      <c r="I30" s="23" t="s">
+        <v>110</v>
       </c>
       <c r="J30" s="15">
-        <f t="shared" ref="J30" si="2">(G30*E30)+F30</f>
-        <v>27.96</v>
+        <f t="shared" ref="J30" si="4">(G30*E30)+F30</f>
+        <v>14.38</v>
       </c>
       <c r="K30" s="15"/>
-      <c r="L30" s="18" t="s">
+      <c r="L30" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M30" s="16"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="15">
         <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
         <v>29</v>
       </c>
-      <c r="B31" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="C31" s="24" t="s">
-        <v>124</v>
+      <c r="B31" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>117</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E31" s="15">
-        <v>7.19</v>
+        <v>4.8899999999999997</v>
       </c>
       <c r="F31" s="15"/>
       <c r="G31" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H31" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I31" s="25" t="s">
-        <v>125</v>
+      <c r="I31" s="23" t="s">
+        <v>115</v>
       </c>
       <c r="J31" s="15">
-        <f t="shared" ref="J31" si="3">(G31*E31)+F31</f>
-        <v>14.38</v>
+        <f t="shared" ref="J31" si="5">(G31*E31)+F31</f>
+        <v>4.8899999999999997</v>
       </c>
       <c r="K31" s="15"/>
-      <c r="L31" s="18" t="s">
+      <c r="L31" s="28" t="s">
         <v>36</v>
       </c>
       <c r="M31" s="16"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
-        <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
-        <v>30</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="C32" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E32" s="15">
-        <v>7.19</v>
-      </c>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15">
-        <v>2</v>
-      </c>
-      <c r="H32" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I32" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="J32" s="15">
-        <f t="shared" ref="J32" si="4">(G32*E32)+F32</f>
-        <v>14.38</v>
-      </c>
-      <c r="K32" s="15"/>
-      <c r="L32" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="M32" s="16"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
-        <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
-        <v>31</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="C33" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E33" s="15">
-        <v>4.8899999999999997</v>
-      </c>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15">
-        <v>1</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I33" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="J33" s="15">
-        <f t="shared" ref="J33" si="5">(G33*E33)+F33</f>
-        <v>4.8899999999999997</v>
-      </c>
-      <c r="K33" s="15"/>
-      <c r="L33" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="M33" s="16"/>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="L32" s="28"/>
+    </row>
+    <row r="33" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L33" s="28"/>
+    </row>
+    <row r="34" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L34" s="28"/>
+    </row>
+    <row r="35" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L35" s="28"/>
+    </row>
+    <row r="36" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L36" s="28"/>
+    </row>
+    <row r="37" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L37" s="28"/>
+    </row>
+    <row r="38" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L38" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="F7:F8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="L3">
-    <cfRule type="expression" priority="1">
+  <conditionalFormatting sqref="L10:L38 L3:L6">
+    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L3)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7">
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L33">
-    <cfRule type="expression" priority="3">
+  <conditionalFormatting sqref="L4:L38">
+    <cfRule type="expression" priority="9">
       <formula>#REF!="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L38">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="approved">
+      <formula>NOT(ISERROR(SEARCH("approved",L3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="ordered">
+      <formula>NOT(ISERROR(SEARCH("ordered",L3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="rejected">
+      <formula>NOT(ISERROR(SEARCH("rejected",L3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="received">
+      <formula>NOT(ISERROR(SEARCH("received",L3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L8:L9">
+    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L8)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13">
+      <formula>#REF!="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7">
+    <cfRule type="containsText" dxfId="1" priority="16" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L7)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17">
+      <formula>$B5="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L6">
+    <cfRule type="containsText" dxfId="0" priority="18" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L6)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19">
+      <formula>$B7="approved"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1" display="https://3dprintx.bg/magazin/pa6-cf-with-spool-cherno-bambu-lab/?gad_source=1&amp;gad_campaignid=23369295043&amp;gbraid=0AAAABBeApTZEPbIRHor7bJZ92Gq7vT3lv&amp;gclid=CjwKCAjwxITRBhBYEiwA6mZm7bCe5kvsvoz_znE0dv8i7YoYQrUSTdOaCQ7RKckeGywr-XLrI4hECRoCo7MQAvD_BwE" xr:uid="{45F219EB-CA0E-46B2-B5AC-321500547349}"/>
-    <hyperlink ref="N11" r:id="rId2" xr:uid="{768681FA-3135-41DB-AF87-7EDFDCB42E31}"/>
+    <hyperlink ref="N9" r:id="rId2" xr:uid="{768681FA-3135-41DB-AF87-7EDFDCB42E31}"/>
+    <hyperlink ref="I5" r:id="rId3" xr:uid="{29AE6930-3CFD-49FA-8C77-A431B4331D49}"/>
+    <hyperlink ref="I6" r:id="rId4" xr:uid="{3002E511-E2F5-4C78-B094-E6DD7CF3B671}"/>
+    <hyperlink ref="I7" r:id="rId5" xr:uid="{46C8B073-4590-4C63-B6E5-2A03FB1E94E6}"/>
+    <hyperlink ref="I8" r:id="rId6" xr:uid="{7085C41A-4F68-4A70-A26C-EBBC546A59EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -2420,19 +2563,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D33</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D191F27-4E1E-4078-9DF4-BD7DE8468C2E}">
-          <x14:formula1>
-            <xm:f>Background_info!$B$3:$B$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>H3:H33</xm:sqref>
+          <xm:sqref>D3:D31</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L33</xm:sqref>
+          <xm:sqref>L3:L38</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4580CAC9-FAF7-403B-A1D9-84CB43CB97A9}">
+          <x14:formula1>
+            <xm:f>Background_info!$B$3:$B$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>H3:H31</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2443,10 +2586,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19"/>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Wing Assembly updates - connection pins
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\P01\P01_06_Procurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13665E8A-36D8-4D5F-9F02-AD80E8FAB20D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E13ACD1-9165-489F-AF15-8A00537D9457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
@@ -667,17 +667,17 @@
     <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1359,7 +1359,7 @@
         <v>127</v>
       </c>
       <c r="L5" s="26" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M5" s="19" t="s">
         <v>123</v>
@@ -1402,7 +1402,7 @@
         <v>130</v>
       </c>
       <c r="L6" s="26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M6" s="19" t="s">
         <v>131</v>
@@ -1425,7 +1425,7 @@
       <c r="E7" s="15">
         <v>31.22</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="30">
         <v>18.75</v>
       </c>
       <c r="G7" s="15">
@@ -1468,7 +1468,7 @@
       <c r="E8" s="15">
         <v>12.83</v>
       </c>
-      <c r="F8" s="29"/>
+      <c r="F8" s="31"/>
       <c r="G8" s="15">
         <v>2</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>48</v>
       </c>
       <c r="L9" s="26" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M9" s="19" t="s">
         <v>120</v>
@@ -1576,7 +1576,7 @@
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="29" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -1660,7 +1660,7 @@
         <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
         <v>11</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="29" t="s">
         <v>56</v>
       </c>
       <c r="C13" s="13" t="s">
@@ -1726,7 +1726,7 @@
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
         <v>13</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="29" t="s">
         <v>53</v>
       </c>
       <c r="C15" s="13" t="s">
@@ -1767,7 +1767,7 @@
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
         <v>14</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="29" t="s">
         <v>69</v>
       </c>
       <c r="C16" s="13" t="s">
@@ -1843,7 +1843,7 @@
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
         <v>16</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="29" t="s">
         <v>79</v>
       </c>
       <c r="C18" s="13" t="s">
@@ -2087,7 +2087,7 @@
         <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
         <v>22</v>
       </c>
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="28" t="s">
         <v>93</v>
       </c>
       <c r="C24" s="13" t="s">
@@ -2130,7 +2130,7 @@
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
       </c>
-      <c r="B25" s="30" t="s">
+      <c r="B25" s="28" t="s">
         <v>66</v>
       </c>
       <c r="C25" s="13" t="s">
@@ -2171,7 +2171,7 @@
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
       </c>
-      <c r="B26" s="30" t="s">
+      <c r="B26" s="28" t="s">
         <v>63</v>
       </c>
       <c r="C26" s="13" t="s">

</xml_diff>